<commit_message>
docs: update feature test results
</commit_message>
<xml_diff>
--- a/docs/testing/test-results.xlsx
+++ b/docs/testing/test-results.xlsx
@@ -31,7 +31,7 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
@@ -41,16 +41,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00D9EAF7"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00D9EAD3"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00E6E6E6"/>
       </patternFill>
     </fill>
   </fills>
@@ -66,18 +56,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -454,10 +438,10 @@
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="18" customWidth="1" min="6" max="6"/>
-    <col width="48" customWidth="1" min="7" max="7"/>
-    <col width="60" customWidth="1" min="8" max="8"/>
-    <col width="48" customWidth="1" min="9" max="9"/>
-    <col width="52" customWidth="1" min="10" max="10"/>
+    <col width="44" customWidth="1" min="7" max="7"/>
+    <col width="58" customWidth="1" min="8" max="8"/>
+    <col width="44" customWidth="1" min="9" max="9"/>
+    <col width="58" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -528,7 +512,7 @@
           <t>Offline</t>
         </is>
       </c>
-      <c r="D2" s="3" t="inlineStr">
+      <c r="D2" s="2" t="inlineStr">
         <is>
           <t>Passed</t>
         </is>
@@ -580,14 +564,14 @@
           <t>Offline</t>
         </is>
       </c>
-      <c r="D3" s="3" t="inlineStr">
+      <c r="D3" s="2" t="inlineStr">
         <is>
           <t>Passed</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
@@ -597,20 +581,24 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>ADAPTISEQ_NO_NETWORK=1 python -m pytest tests/test_segmented.py tests/test_segmented_finalize.py -q</t>
+          <t>ADAPTISEQ_NO_NETWORK=1 python -m pytest tests/test_segmented.py tests/test_ftp_segmented.py -q</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>23 passed</t>
+          <t>27 passed</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>User-reported terminal output</t>
-        </is>
-      </c>
-      <c r="J3" s="2" t="inlineStr"/>
+          <t>Codex-run pytest output</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>Rerun after display-interval changes; local socket tests required sandbox escalation; earlier finalize coverage remained passed</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -628,14 +616,14 @@
           <t>Offline</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="D4" s="2" t="inlineStr">
         <is>
           <t>Passed</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
@@ -645,17 +633,17 @@
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>ADAPTISEQ_NO_NETWORK=1 python -m pytest tests/test_ftp_segmented.py -q</t>
+          <t>ADAPTISEQ_NO_NETWORK=1 python -m pytest tests/test_segmented.py tests/test_ftp_segmented.py -q</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>3 passed</t>
+          <t>Included in combined 27 passed rerun</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>User-reported terminal output</t>
+          <t>Codex-run pytest output</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr"/>
@@ -676,14 +664,14 @@
           <t>Offline</t>
         </is>
       </c>
-      <c r="D5" s="3" t="inlineStr">
+      <c r="D5" s="2" t="inlineStr">
         <is>
           <t>Passed</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
@@ -698,7 +686,7 @@
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>22 passed</t>
+          <t>23 passed</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
@@ -708,7 +696,7 @@
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>Includes worker-cap and success-log regression coverage; loopback server tests require local socket permission</t>
+          <t>Includes worker-cap, display interval, and success-log regression coverage; loopback server tests require local socket permission</t>
         </is>
       </c>
     </row>
@@ -728,7 +716,7 @@
           <t>Offline</t>
         </is>
       </c>
-      <c r="D6" s="3" t="inlineStr">
+      <c r="D6" s="2" t="inlineStr">
         <is>
           <t>Passed</t>
         </is>
@@ -776,7 +764,7 @@
           <t>Offline</t>
         </is>
       </c>
-      <c r="D7" s="3" t="inlineStr">
+      <c r="D7" s="2" t="inlineStr">
         <is>
           <t>Passed</t>
         </is>
@@ -828,14 +816,14 @@
           <t>Offline</t>
         </is>
       </c>
-      <c r="D8" s="3" t="inlineStr">
+      <c r="D8" s="2" t="inlineStr">
         <is>
           <t>Passed</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
@@ -880,7 +868,7 @@
           <t>Live</t>
         </is>
       </c>
-      <c r="D9" s="3" t="inlineStr">
+      <c r="D9" s="2" t="inlineStr">
         <is>
           <t>Passed</t>
         </is>
@@ -928,7 +916,7 @@
           <t>Live</t>
         </is>
       </c>
-      <c r="D10" s="3" t="inlineStr">
+      <c r="D10" s="2" t="inlineStr">
         <is>
           <t>Passed</t>
         </is>
@@ -976,7 +964,7 @@
           <t>Live</t>
         </is>
       </c>
-      <c r="D11" s="3" t="inlineStr">
+      <c r="D11" s="2" t="inlineStr">
         <is>
           <t>Passed</t>
         </is>
@@ -1024,7 +1012,7 @@
           <t>Live</t>
         </is>
       </c>
-      <c r="D12" s="3" t="inlineStr">
+      <c r="D12" s="2" t="inlineStr">
         <is>
           <t>Passed</t>
         </is>
@@ -1076,7 +1064,7 @@
           <t>Live</t>
         </is>
       </c>
-      <c r="D13" s="3" t="inlineStr">
+      <c r="D13" s="2" t="inlineStr">
         <is>
           <t>Passed</t>
         </is>
@@ -1128,7 +1116,7 @@
           <t>Live</t>
         </is>
       </c>
-      <c r="D14" s="3" t="inlineStr">
+      <c r="D14" s="2" t="inlineStr">
         <is>
           <t>Passed</t>
         </is>
@@ -1180,7 +1168,7 @@
           <t>Live</t>
         </is>
       </c>
-      <c r="D15" s="3" t="inlineStr">
+      <c r="D15" s="2" t="inlineStr">
         <is>
           <t>Passed</t>
         </is>
@@ -1232,7 +1220,7 @@
           <t>Live</t>
         </is>
       </c>
-      <c r="D16" s="3" t="inlineStr">
+      <c r="D16" s="2" t="inlineStr">
         <is>
           <t>Passed</t>
         </is>
@@ -1284,7 +1272,7 @@
           <t>Live</t>
         </is>
       </c>
-      <c r="D17" s="3" t="inlineStr">
+      <c r="D17" s="2" t="inlineStr">
         <is>
           <t>Passed</t>
         </is>
@@ -1336,7 +1324,7 @@
           <t>Live</t>
         </is>
       </c>
-      <c r="D18" s="3" t="inlineStr">
+      <c r="D18" s="2" t="inlineStr">
         <is>
           <t>Passed</t>
         </is>
@@ -1388,7 +1376,7 @@
           <t>Live</t>
         </is>
       </c>
-      <c r="D19" s="3" t="inlineStr">
+      <c r="D19" s="2" t="inlineStr">
         <is>
           <t>Passed</t>
         </is>
@@ -1440,7 +1428,7 @@
           <t>Live</t>
         </is>
       </c>
-      <c r="D20" s="3" t="inlineStr">
+      <c r="D20" s="2" t="inlineStr">
         <is>
           <t>Passed</t>
         </is>
@@ -1492,7 +1480,7 @@
           <t>Live</t>
         </is>
       </c>
-      <c r="D21" s="3" t="inlineStr">
+      <c r="D21" s="2" t="inlineStr">
         <is>
           <t>Passed</t>
         </is>
@@ -1544,23 +1532,39 @@
           <t>Live</t>
         </is>
       </c>
-      <c r="D22" s="4" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="E22" s="2" t="inlineStr"/>
-      <c r="F22" s="2" t="inlineStr"/>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>Conda adaptiseq</t>
+        </is>
+      </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
           <t>adaptiseq -i SRR1178105 -q -t 2 -o tmp/feature-tests/tc14</t>
         </is>
       </c>
-      <c r="H22" s="2" t="inlineStr"/>
-      <c r="I22" s="2" t="inlineStr"/>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t>Completed successfully; downloaded SRR1178105 at 291744155 bytes, verified md5, converted with fasterq-dump -t 2, and wrote paired FASTQ files; each FASTQ has 10044848 lines, matching 2511212 reads per mate</t>
+        </is>
+      </c>
+      <c r="I22" s="2" t="inlineStr">
+        <is>
+          <t>tmp/feature-tests/tc14/success.log; tmp/feature-tests/tc14/SRR1178105_1.fastq; tmp/feature-tests/tc14/SRR1178105_2.fastq</t>
+        </is>
+      </c>
       <c r="J22" s="2" t="inlineStr">
         <is>
-          <t>Requires srapath; fasterq-dump; vdb-validate; pigz</t>
+          <t>success.log contains SRR1178105; each FASTQ is 698694944 bytes; no fail.log exists; logging behavior is expected because file progress, segment meters, and adaptive probes use separate intervals</t>
         </is>
       </c>
     </row>
@@ -1580,7 +1584,7 @@
           <t>Live</t>
         </is>
       </c>
-      <c r="D23" s="4" t="inlineStr">
+      <c r="D23" s="2" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -1612,23 +1616,39 @@
           <t>Live</t>
         </is>
       </c>
-      <c r="D24" s="4" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="E24" s="2" t="inlineStr"/>
-      <c r="F24" s="2" t="inlineStr"/>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>Conda adaptiseq</t>
+        </is>
+      </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
           <t>adaptiseq -i SRR7706354 -e ex -o tmp/feature-tests/tc16</t>
         </is>
       </c>
-      <c r="H24" s="2" t="inlineStr"/>
-      <c r="I24" s="2" t="inlineStr"/>
+      <c r="H24" s="2" t="inlineStr">
+        <is>
+          <t>Exited with expected guard error: SRR7706354 is a Run ID, can not use -e option; printed expected solution text</t>
+        </is>
+      </c>
+      <c r="I24" s="2" t="inlineStr">
+        <is>
+          <t>No artifacts created</t>
+        </is>
+      </c>
       <c r="J24" s="2" t="inlineStr">
         <is>
-          <t>Expected non-zero exit</t>
+          <t>Expected non-zero exit before download</t>
         </is>
       </c>
     </row>
@@ -1648,7 +1668,7 @@
           <t>Live</t>
         </is>
       </c>
-      <c r="D25" s="4" t="inlineStr">
+      <c r="D25" s="2" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -1680,7 +1700,7 @@
           <t>Live</t>
         </is>
       </c>
-      <c r="D26" s="4" t="inlineStr">
+      <c r="D26" s="2" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -1716,7 +1736,7 @@
           <t>Live</t>
         </is>
       </c>
-      <c r="D27" s="4" t="inlineStr">
+      <c r="D27" s="2" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -1752,7 +1772,7 @@
           <t>Live</t>
         </is>
       </c>
-      <c r="D28" s="4" t="inlineStr">
+      <c r="D28" s="2" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -1784,7 +1804,7 @@
           <t>Live</t>
         </is>
       </c>
-      <c r="D29" s="4" t="inlineStr">
+      <c r="D29" s="2" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>

</xml_diff>

<commit_message>
docs: record skip-md5 feature test
</commit_message>
<xml_diff>
--- a/docs/testing/test-results.xlsx
+++ b/docs/testing/test-results.xlsx
@@ -1670,19 +1670,39 @@
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="E25" s="2" t="inlineStr"/>
-      <c r="F25" s="2" t="inlineStr"/>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>Conda adaptiseq</t>
+        </is>
+      </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
           <t>adaptiseq -i SRR22904257 -g -r https -k --engine segmented -o tmp/feature-tests/tc17</t>
         </is>
       </c>
-      <c r="H25" s="2" t="inlineStr"/>
-      <c r="I25" s="2" t="inlineStr"/>
-      <c r="J25" s="2" t="inlineStr"/>
+      <c r="H25" s="2" t="inlineStr">
+        <is>
+          <t>Completed successfully and printed Skip md5 check for SRR22904257, as -k option is used</t>
+        </is>
+      </c>
+      <c r="I25" s="2" t="inlineStr">
+        <is>
+          <t>tmp/feature-tests/tc17/SRR22904257.fastq.gz; tmp/feature-tests/tc17/SRR22904257.metadata.tsv</t>
+        </is>
+      </c>
+      <c r="J25" s="2" t="inlineStr">
+        <is>
+          <t>FASTQ gzip is 50963 bytes; no fail.log exists; success.log is empty because this mode skips verification rather than recording an md5-verified success</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">

</xml_diff>

<commit_message>
fix: normalize ENA aspera links
</commit_message>
<xml_diff>
--- a/docs/testing/test-results.xlsx
+++ b/docs/testing/test-results.xlsx
@@ -1722,21 +1722,37 @@
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="E26" s="2" t="inlineStr"/>
-      <c r="F26" s="2" t="inlineStr"/>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>Conda adaptiseq</t>
+        </is>
+      </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
           <t>adaptiseq -i SRR22904257 -a -g --aspera-efficiency 0.70 -o tmp/feature-tests/tc18</t>
         </is>
       </c>
-      <c r="H26" s="2" t="inlineStr"/>
-      <c r="I26" s="2" t="inlineStr"/>
+      <c r="H26" s="2" t="inlineStr">
+        <is>
+          <t>Live run reached real ascp but failed with failed to authenticate; no FASTQ was downloaded and fail.log recorded SRR22904257; root cause was ENA fastq_aspera metadata in fasp.sra.ebi.ac.uk:/... form being passed without era-fasp@ user</t>
+        </is>
+      </c>
+      <c r="I26" s="2" t="inlineStr">
+        <is>
+          <t>tmp/feature-tests/tc18/fail.log</t>
+        </is>
+      </c>
       <c r="J26" s="2" t="inlineStr">
         <is>
-          <t>Requires real IBM ascp</t>
+          <t>Code now normalizes ENA Aspera links to era-fasp@fasp.sra.ebi.ac.uk:/... and focused tests pass; rerun TC-18 from this revision to confirm live transfer</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: mark ENA aspera test blocked
</commit_message>
<xml_diff>
--- a/docs/testing/test-results.xlsx
+++ b/docs/testing/test-results.xlsx
@@ -1722,7 +1722,7 @@
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>Partial</t>
+          <t>Blocked</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
@@ -1742,7 +1742,7 @@
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>Live run reached real ascp but failed with failed to authenticate; no FASTQ was downloaded and fail.log recorded SRR22904257; root cause was ENA fastq_aspera metadata in fasp.sra.ebi.ac.uk:/... form being passed without era-fasp@ user</t>
+          <t>Live adaptiSeq run and direct ascp probes both failed with failed to authenticate; ENA key is found and was changed to 0600; adaptiSeq now normalizes target to era-fasp@fasp.sra.ebi.ac.uk:... but standalone Aspera client still cannot authenticate to ENA</t>
         </is>
       </c>
       <c r="I26" s="2" t="inlineStr">
@@ -1752,7 +1752,7 @@
       </c>
       <c r="J26" s="2" t="inlineStr">
         <is>
-          <t>Code now normalizes ENA Aspera links to era-fasp@fasp.sra.ebi.ac.uk:/... and focused tests pass; rerun TC-18 from this revision to confirm live transfer</t>
+          <t>Blocked by external Aspera authentication/key compatibility, not adaptiSeq command construction; use HTTPS/FTP tests for this accession until ENA Aspera credentials/client are resolved</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: record TC-22..TC-28 results — all passed
Ran the seven new cases in the Conda adaptiseq env; all passed:
- TC-22 GSE122139 -> PRJNA503819 (GEO Series resolution)
- TC-23 GSM7417667 -> SAMN35350598 -> SRR24721990 paired, md5 OK (GEO Sample)
- TC-24 CRR311377 483 MB via segmented FTP, md5 OK (GSA data download)
- TC-25/26 SAMC017083 / PRJCA000613 -> CRR022335+CRR022336 merged (GSA -e sa/st)
- TC-27 DRR421224 ~746 MB via ENA mirror, md5 OK (DDBJ run)
- TC-28 PRJDB14838 -> 6 DDBJ runs ~3.7 GB via adaptive batch pool, md5 OK

Summary: Passed 33, Failed 0, Blocked 2 (Aspera TC-18/TC-19, external), Not Run 0.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/testing/test-results.xlsx
+++ b/docs/testing/test-results.xlsx
@@ -422,7 +422,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J29"/>
+  <dimension ref="A1:J36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1925,6 +1925,370 @@
         </is>
       </c>
     </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>TC-22</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>GEO Series Resolution (GSE)</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>Live</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="inlineStr">
+        <is>
+          <t>Conda adaptiseq</t>
+        </is>
+      </c>
+      <c r="G30" s="2" t="inlineStr">
+        <is>
+          <t>adaptiseq -i GSE122139 -m -o tmp/feature-tests/tc22</t>
+        </is>
+      </c>
+      <c r="H30" s="2" t="inlineStr">
+        <is>
+          <t>Printed 'GSE122139 belongs to PRJNA503819'; wrote GSE122139.metadata.tsv (metadata only); resolved on first attempt</t>
+        </is>
+      </c>
+      <c r="I30" s="2" t="inlineStr">
+        <is>
+          <t>tmp/feature-tests/tc22/GSE122139.metadata.tsv</t>
+        </is>
+      </c>
+      <c r="J30" s="2" t="inlineStr">
+        <is>
+          <t>Validates GEO Series -&gt; BioProject resolution</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>TC-23</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>GEO Sample Download (GSM)</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>Live</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="F31" s="2" t="inlineStr">
+        <is>
+          <t>Conda adaptiseq</t>
+        </is>
+      </c>
+      <c r="G31" s="2" t="inlineStr">
+        <is>
+          <t>adaptiseq -i GSM7417667 -g -r https -o tmp/feature-tests/tc23</t>
+        </is>
+      </c>
+      <c r="H31" s="2" t="inlineStr">
+        <is>
+          <t>GSM7417667 -&gt; SAMN35350598 -&gt; run SRR24721990 PAIRED; SRR24721990_1.fastq.gz 65.75 MB + _2.fastq.gz 68.38 MB via segmented HTTPS, md5 OK, in success.log</t>
+        </is>
+      </c>
+      <c r="I31" s="2" t="inlineStr">
+        <is>
+          <t>tmp/feature-tests/tc23/</t>
+        </is>
+      </c>
+      <c r="J31" s="2" t="inlineStr">
+        <is>
+          <t>No fail.log; validates GEO Sample -&gt; BioSample resolution + download</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>TC-24</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>GSA Sequence-Data Download</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>Live</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t>Conda adaptiseq</t>
+        </is>
+      </c>
+      <c r="G32" s="2" t="inlineStr">
+        <is>
+          <t>adaptiseq -i CRR311377 -g -o tmp/feature-tests/tc24</t>
+        </is>
+      </c>
+      <c r="H32" s="2" t="inlineStr">
+        <is>
+          <t>CRR311377 (GSA, CRA004720) downloaded CRR311377.fq.gz 483 MB; Database GSA Mode ftp; download.big.ac.cn supports REST+concurrency so used native segmented FTP; md5 OK, in success.log</t>
+        </is>
+      </c>
+      <c r="I32" s="2" t="inlineStr">
+        <is>
+          <t>tmp/feature-tests/tc24/</t>
+        </is>
+      </c>
+      <c r="J32" s="2" t="inlineStr">
+        <is>
+          <t>Fills GSA data path vs metadata-only TC-03; Huawei-priority still not exercised (no huaweicloud link)</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>TC-25</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>Merge by Sample (-e sa, GSA)</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>Live</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="F33" s="2" t="inlineStr">
+        <is>
+          <t>Conda adaptiseq</t>
+        </is>
+      </c>
+      <c r="G33" s="2" t="inlineStr">
+        <is>
+          <t>adaptiseq -i SAMC017083 -g -e sa -o tmp/feature-tests/tc25</t>
+        </is>
+      </c>
+      <c r="H33" s="2" t="inlineStr">
+        <is>
+          <t>SAMC017083 -&gt; CRA000553; CRR022335.fastq.gz 579 MB + CRR022336.fastq.gz 437 MB via segmented FTP, both md5 OK in success.log; merged into SAMC017083.fastq.gz</t>
+        </is>
+      </c>
+      <c r="I33" s="2" t="inlineStr">
+        <is>
+          <t>tmp/feature-tests/tc25/</t>
+        </is>
+      </c>
+      <c r="J33" s="2" t="inlineStr">
+        <is>
+          <t>GSA merge-by-Sample works (merge_gsa_run); mirrors iSeq SAMC017083 -e sa</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>TC-26</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>Merge by Study (-e st, GSA)</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>Live</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="F34" s="2" t="inlineStr">
+        <is>
+          <t>Conda adaptiseq</t>
+        </is>
+      </c>
+      <c r="G34" s="2" t="inlineStr">
+        <is>
+          <t>adaptiseq -i PRJCA000613 -g -e st -o tmp/feature-tests/tc26</t>
+        </is>
+      </c>
+      <c r="H34" s="2" t="inlineStr">
+        <is>
+          <t>PRJCA000613 -&gt; CRA000553; same 2 runs CRR022335 579 MB + CRR022336 437 MB via segmented FTP, md5 OK; merged into PRJCA000613.fastq.gz</t>
+        </is>
+      </c>
+      <c r="I34" s="2" t="inlineStr">
+        <is>
+          <t>tmp/feature-tests/tc26/</t>
+        </is>
+      </c>
+      <c r="J34" s="2" t="inlineStr">
+        <is>
+          <t>GSA merge-by-Study + Project fan-out works; mirrors iSeq PRJCA000613 -e st</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>TC-27</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>DDBJ Run Download</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>Live</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="F35" s="2" t="inlineStr">
+        <is>
+          <t>Conda adaptiseq</t>
+        </is>
+      </c>
+      <c r="G35" s="2" t="inlineStr">
+        <is>
+          <t>adaptiseq -i DRR421224 -g -r https -o tmp/feature-tests/tc27</t>
+        </is>
+      </c>
+      <c r="H35" s="2" t="inlineStr">
+        <is>
+          <t>DDBJ run DRR421224 via segmented HTTPS (ftp.sra.ebi.ac.uk, ~746 MB, Database ENA Mode https), md5 OK in success.log; 14 adaptive probes held at 1 worker (best 74 Mbps)</t>
+        </is>
+      </c>
+      <c r="I35" s="2" t="inlineStr">
+        <is>
+          <t>tmp/feature-tests/tc27/</t>
+        </is>
+      </c>
+      <c r="J35" s="2" t="inlineStr">
+        <is>
+          <t>DDBJ live path works; run served via ENA mirror; previously offline/parity only</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>TC-28</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>Project/Study Live Download</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>Live</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="F36" s="2" t="inlineStr">
+        <is>
+          <t>Conda adaptiseq</t>
+        </is>
+      </c>
+      <c r="G36" s="2" t="inlineStr">
+        <is>
+          <t>adaptiseq -i PRJDB14838 -g -r https -o tmp/feature-tests/tc28</t>
+        </is>
+      </c>
+      <c r="H36" s="2" t="inlineStr">
+        <is>
+          <t>DDBJ Project PRJDB14838 -&gt; 6 runs DRR421222-DRR421227 (~3.7 GB) all via segmented HTTPS (Database ENA Mode https), md5 OK, all 6 in success.log; adaptive pool ran 34 probes scaling 1-3 workers (best 148 Mbps)</t>
+        </is>
+      </c>
+      <c r="I36" s="2" t="inlineStr">
+        <is>
+          <t>tmp/feature-tests/tc28/</t>
+        </is>
+      </c>
+      <c r="J36" s="2" t="inlineStr">
+        <is>
+          <t>Project fan-out + adaptive batch pool on a real multi-file project; DDBJ via ENA mirror</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
docs: corroborate TC-18/TC-19 Aspera blockers with upstream iseq cross-check
Cloned BioOmics/iSeq (the original Bash tool) and ran the two blocked
accessions with the same conda toolchain. Both fail identically to adaptiSeq,
confirming the blockers are external (not adaptiSeq defects):
- TC-18 ENA Aspera SRR22904257: iseq -> 'ascp: failed to authenticate' x3 ->
  fail.log, using the same RSA key (aspera_bypass_rsa.pem) and ascp command.
- TC-19 GSA Aspera CRR343031: iseq -> 'Failed to open TCP connection for SSH';
  f1 downloaded (1.67 GB, md5 OK), r2 failed all 3 retries -> fail.log; same
  intermittent/partial pattern, same ascp command/endpoint.

Added the cross-check to the TC-18/TC-19 notes in the .md/.csv/.xlsx report.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/testing/test-results.xlsx
+++ b/docs/testing/test-results.xlsx
@@ -1765,7 +1765,7 @@
       </c>
       <c r="J26" s="2" t="inlineStr">
         <is>
-          <t>Blocked by external Aspera authentication/key compatibility, not adaptiSeq command construction; use HTTPS/FTP tests for this accession until ENA Aspera credentials/client are resolved</t>
+          <t>Blocked by external Aspera authentication/key compatibility, not adaptiSeq command construction; use HTTPS/FTP tests for this accession until ENA Aspera credentials/client are resolved. Cross-checked 2026-06-28: upstream BioOmics/iSeq with the same conda toolchain fails identically (ascp failed to authenticate x3 -&gt; fail.log) using the same RSA key and ascp command - confirms external blocker not adaptiSeq-specific</t>
         </is>
       </c>
     </row>
@@ -1817,7 +1817,7 @@
       </c>
       <c r="J27" s="2" t="inlineStr">
         <is>
-          <t>Not an adaptiSeq defect - f1 completing proves endpoint/key/command/routing are correct (not auth, unlike TC-18). Probable cause: long-haul international path to GSA host download.cncb.ac.cn (NGDC Beijing); Aspera needs both a TCP/SSH control channel and a UDP data channel on port 33001 and both intermittently fail (TCP control handshake dropped; UDP data blocked/lossy) - likely packet loss, an institutional firewall filtering/rate-limiting TCP+UDP 33001, or per-IP connection limits. Mitigations: re-run (only r2 retries; f1 skipped via success.log) or drop -a for GSA https/ftp (no UDP). Huawei-first branch not exercised because CRR343031 has no huaweicloud links</t>
+          <t>Not an adaptiSeq defect - f1 completing proves endpoint/key/command/routing are correct (not auth, unlike TC-18). Probable cause: long-haul international path to GSA host download.cncb.ac.cn (NGDC Beijing); Aspera needs both a TCP/SSH control channel and a UDP data channel on port 33001 and both intermittently fail (TCP control handshake dropped; UDP data blocked/lossy) - likely packet loss, an institutional firewall filtering/rate-limiting TCP+UDP 33001, or per-IP connection limits. Mitigations: re-run (only r2 retries; f1 skipped via success.log) or drop -a for GSA https/ftp (no UDP). Huawei-first branch not exercised because CRR343031 has no huaweicloud links. Cross-checked 2026-06-28: upstream iseq reproduces the same intermittent/partial result (Failed to open TCP connection for SSH; f1 downloaded 1.67 GB md5 OK, r2 failed 3 retries -&gt; fail.log) with the same ascp command/endpoint - confirms external not adaptiSeq-specific</t>
         </is>
       </c>
     </row>

</xml_diff>